<commit_message>
partidos, sin datos, descarga, codebook
</commit_message>
<xml_diff>
--- a/data/dictionary.xlsx
+++ b/data/dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pipei\OneDrive\Escritorio\subn_v3\subnational_gov\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD1EE2D8-F125-4AB2-83E8-F3C5B054DF3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5AF2356-F7DF-4A11-8EEA-88F8BB118EF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="240">
   <si>
     <t>country_name</t>
   </si>
@@ -756,13 +756,16 @@
   </si>
   <si>
     <t>#ff8000,#00E5FF</t>
+  </si>
+  <si>
+    <t>#1f77b4,#ff7f0e,#2ca02c,#d62728,#9467bd,#e377c2,#8c564b,#bcbd22,#17becf,#aec7e8,#ffbb78,#98df8a,#d95f02</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -772,6 +775,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -799,9 +810,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1082,8 +1097,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.85546875" bestFit="1" customWidth="1"/>
@@ -1091,6 +1105,7 @@
     <col min="4" max="4" width="85.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1119,7 +1134,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1142,7 +1157,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -1165,7 +1180,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1188,7 +1203,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1211,7 +1226,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -1260,7 +1275,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -1283,7 +1298,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
@@ -1361,7 +1376,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -1384,7 +1399,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -1436,7 +1451,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>24</v>
       </c>
@@ -1485,7 +1500,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>28</v>
       </c>
@@ -1508,7 +1523,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -1534,7 +1549,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -1560,7 +1575,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>34</v>
       </c>
@@ -1586,7 +1601,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -1612,7 +1627,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>38</v>
       </c>
@@ -1638,7 +1653,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>40</v>
       </c>
@@ -1664,7 +1679,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>42</v>
       </c>
@@ -1680,14 +1695,18 @@
       <c r="E24" t="s">
         <v>161</v>
       </c>
+      <c r="F24" t="s">
+        <v>239</v>
+      </c>
       <c r="G24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H24" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K24" s="2"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>44</v>
       </c>
@@ -1703,7 +1722,7 @@
       <c r="E25" t="s">
         <v>163</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="3" t="s">
         <v>238</v>
       </c>
       <c r="G25">
@@ -1713,7 +1732,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>46</v>
       </c>
@@ -1739,7 +1758,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>48</v>
       </c>
@@ -1765,7 +1784,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>50</v>
       </c>
@@ -1791,7 +1810,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>52</v>
       </c>
@@ -1817,7 +1836,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>54</v>
       </c>
@@ -1843,7 +1862,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>56</v>
       </c>
@@ -1869,7 +1888,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>58</v>
       </c>
@@ -1921,7 +1940,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>62</v>
       </c>
@@ -1944,7 +1963,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>64</v>
       </c>
@@ -1970,7 +1989,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>66</v>
       </c>
@@ -1996,7 +2015,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>68</v>
       </c>
@@ -2022,7 +2041,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>70</v>
       </c>
@@ -2048,7 +2067,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>72</v>
       </c>
@@ -2074,7 +2093,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>74</v>
       </c>
@@ -2100,7 +2119,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>76</v>
       </c>
@@ -2126,7 +2145,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>78</v>
       </c>
@@ -2152,7 +2171,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>80</v>
       </c>
@@ -2178,7 +2197,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>82</v>
       </c>
@@ -2204,7 +2223,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>84</v>
       </c>
@@ -2230,7 +2249,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>86</v>
       </c>
@@ -2256,7 +2275,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>88</v>
       </c>
@@ -2282,7 +2301,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>90</v>
       </c>
@@ -2308,7 +2327,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>92</v>
       </c>
@@ -2334,7 +2353,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>94</v>
       </c>
@@ -2360,7 +2379,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>96</v>
       </c>
@@ -2380,7 +2399,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>98</v>
       </c>
@@ -2397,7 +2416,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>100</v>
       </c>
@@ -2414,7 +2433,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>102</v>
       </c>
@@ -2431,7 +2450,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>104</v>
       </c>
@@ -2451,7 +2470,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>106</v>
       </c>
@@ -2468,7 +2487,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>108</v>
       </c>
@@ -2488,7 +2507,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>110</v>
       </c>
@@ -2505,7 +2524,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>112</v>
       </c>
@@ -2525,7 +2544,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>114</v>
       </c>
@@ -2542,7 +2561,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>116</v>
       </c>
@@ -2562,7 +2581,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>118</v>
       </c>
@@ -2579,7 +2598,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>120</v>
       </c>
@@ -2599,7 +2618,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>122</v>
       </c>
@@ -2616,7 +2635,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>124</v>
       </c>
@@ -2636,7 +2655,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>126</v>
       </c>
@@ -2653,7 +2672,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>128</v>
       </c>
@@ -2673,7 +2692,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>130</v>
       </c>
@@ -2690,7 +2709,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>132</v>
       </c>
@@ -2710,7 +2729,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>134</v>
       </c>
@@ -2727,7 +2746,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>136</v>
       </c>
@@ -2744,7 +2763,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>138</v>
       </c>
@@ -2761,7 +2780,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>140</v>
       </c>
@@ -2781,7 +2800,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>142</v>
       </c>
@@ -2798,7 +2817,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>144</v>
       </c>
@@ -2818,7 +2837,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>146</v>
       </c>
@@ -2835,7 +2854,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>148</v>
       </c>
@@ -2852,7 +2871,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>150</v>
       </c>
@@ -2869,7 +2888,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>152</v>
       </c>
@@ -2886,7 +2905,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>154</v>
       </c>
@@ -2903,7 +2922,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>156</v>
       </c>
@@ -2921,14 +2940,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H81" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="binary"/>
-        <filter val="gender"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:H81" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
fix variables graph y map
</commit_message>
<xml_diff>
--- a/data/dictionary.xlsx
+++ b/data/dictionary.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pipei\OneDrive\Escritorio\subn_v3\subnational_gov\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBC2ADD5-6D0A-40DC-B21A-CFDC2751D9AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A196BFB-9593-461C-BA5D-DCFB8898D7AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-45" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$H$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$I$81</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="241">
   <si>
     <t>country_name</t>
   </si>
@@ -581,9 +581,6 @@
     <t>#efedf5,#bcbddc,#756bb1,#54278f</t>
   </si>
   <si>
-    <t>viewable</t>
-  </si>
-  <si>
     <t>scope</t>
   </si>
   <si>
@@ -759,13 +756,19 @@
   </si>
   <si>
     <t>percentage</t>
+  </si>
+  <si>
+    <t>viewable_map</t>
+  </si>
+  <si>
+    <t>viewable_graph</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -782,6 +785,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <u/>
       <sz val="11"/>
       <color theme="1"/>
@@ -810,13 +822,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1097,24 +1111,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:K81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L81"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="38.88671875" customWidth="1"/>
-    <col min="4" max="4" width="85.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="38.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="38.85546875" customWidth="1"/>
+    <col min="4" max="4" width="85.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>158</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>168</v>
@@ -1128,19 +1141,22 @@
       <c r="F1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C2" t="s">
         <v>169</v>
@@ -1151,19 +1167,22 @@
       <c r="E2" t="s">
         <v>161</v>
       </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="G2" s="5">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C3" t="s">
         <v>169</v>
@@ -1172,21 +1191,24 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
-      <c r="H3" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C4" t="s">
         <v>169</v>
@@ -1200,16 +1222,19 @@
       <c r="G4">
         <v>0</v>
       </c>
-      <c r="H4" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C5" t="s">
         <v>169</v>
@@ -1223,16 +1248,19 @@
       <c r="G5">
         <v>0</v>
       </c>
-      <c r="H5" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C6" t="s">
         <v>169</v>
@@ -1246,16 +1274,19 @@
       <c r="G6">
         <v>0</v>
       </c>
-      <c r="H6" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C7" t="s">
         <v>169</v>
@@ -1264,24 +1295,27 @@
         <v>9</v>
       </c>
       <c r="E7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
-      <c r="H7" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C8" t="s">
         <v>169</v>
@@ -1295,16 +1329,19 @@
       <c r="G8">
         <v>0</v>
       </c>
-      <c r="H8" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C9" t="s">
         <v>169</v>
@@ -1313,7 +1350,7 @@
         <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F9" t="s">
         <v>175</v>
@@ -1321,16 +1358,19 @@
       <c r="G9">
         <v>1</v>
       </c>
-      <c r="H9" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>14</v>
       </c>
       <c r="B10" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C10" t="s">
         <v>169</v>
@@ -1342,21 +1382,24 @@
         <v>163</v>
       </c>
       <c r="F10" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G10">
         <v>1</v>
       </c>
-      <c r="H10" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C11" t="s">
         <v>169</v>
@@ -1368,21 +1411,24 @@
         <v>163</v>
       </c>
       <c r="F11" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G11">
         <v>1</v>
       </c>
-      <c r="H11" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C12" t="s">
         <v>169</v>
@@ -1396,16 +1442,19 @@
       <c r="G12">
         <v>0</v>
       </c>
-      <c r="H12" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C13" t="s">
         <v>169</v>
@@ -1422,16 +1471,19 @@
       <c r="G13">
         <v>1</v>
       </c>
-      <c r="H13" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C14" t="s">
         <v>169</v>
@@ -1443,21 +1495,24 @@
         <v>163</v>
       </c>
       <c r="F14" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G14">
         <v>1</v>
       </c>
-      <c r="H14" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H14">
+        <v>0</v>
+      </c>
+      <c r="I14" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C15" t="s">
         <v>169</v>
@@ -1471,16 +1526,19 @@
       <c r="G15">
         <v>0</v>
       </c>
-      <c r="H15" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>26</v>
       </c>
       <c r="B16" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C16" t="s">
         <v>169</v>
@@ -1489,24 +1547,27 @@
         <v>27</v>
       </c>
       <c r="E16" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F16" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G16">
         <v>1</v>
       </c>
-      <c r="H16" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H16">
+        <v>0</v>
+      </c>
+      <c r="I16" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>28</v>
       </c>
       <c r="B17" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C17" t="s">
         <v>169</v>
@@ -1520,16 +1581,19 @@
       <c r="G17">
         <v>0</v>
       </c>
-      <c r="H17" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H17">
+        <v>0</v>
+      </c>
+      <c r="I17" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>30</v>
       </c>
       <c r="B18" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C18" t="s">
         <v>169</v>
@@ -1541,21 +1605,24 @@
         <v>163</v>
       </c>
       <c r="F18" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G18">
-        <v>1</v>
-      </c>
-      <c r="H18" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H18">
+        <v>0</v>
+      </c>
+      <c r="I18" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>32</v>
       </c>
       <c r="B19" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C19" t="s">
         <v>169</v>
@@ -1564,24 +1631,27 @@
         <v>33</v>
       </c>
       <c r="E19" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F19" t="s">
         <v>175</v>
       </c>
       <c r="G19">
-        <v>1</v>
-      </c>
-      <c r="H19" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
+      <c r="I19" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>34</v>
       </c>
       <c r="B20" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C20" t="s">
         <v>169</v>
@@ -1590,7 +1660,7 @@
         <v>35</v>
       </c>
       <c r="E20" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F20" t="s">
         <v>175</v>
@@ -1598,16 +1668,19 @@
       <c r="G20">
         <v>1</v>
       </c>
-      <c r="H20" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H20">
+        <v>1</v>
+      </c>
+      <c r="I20" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>36</v>
       </c>
       <c r="B21" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C21" t="s">
         <v>169</v>
@@ -1619,21 +1692,24 @@
         <v>163</v>
       </c>
       <c r="F21" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G21">
         <v>1</v>
       </c>
-      <c r="H21" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H21">
+        <v>0</v>
+      </c>
+      <c r="I21" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>38</v>
       </c>
       <c r="B22" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C22" t="s">
         <v>169</v>
@@ -1645,21 +1721,24 @@
         <v>163</v>
       </c>
       <c r="F22" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G22">
         <v>1</v>
       </c>
-      <c r="H22" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H22">
+        <v>0</v>
+      </c>
+      <c r="I22" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>40</v>
       </c>
       <c r="B23" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C23" t="s">
         <v>169</v>
@@ -1668,7 +1747,7 @@
         <v>41</v>
       </c>
       <c r="E23" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F23" t="s">
         <v>175</v>
@@ -1676,16 +1755,19 @@
       <c r="G23">
         <v>1</v>
       </c>
-      <c r="H23" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>42</v>
       </c>
       <c r="B24" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C24" t="s">
         <v>169</v>
@@ -1700,17 +1782,20 @@
       <c r="G24">
         <v>1</v>
       </c>
-      <c r="H24" t="s">
-        <v>184</v>
-      </c>
-      <c r="K24" s="2"/>
-    </row>
-    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24" t="s">
+        <v>183</v>
+      </c>
+      <c r="L24" s="2"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>44</v>
       </c>
       <c r="B25" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C25" t="s">
         <v>169</v>
@@ -1722,21 +1807,24 @@
         <v>163</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G25">
-        <v>1</v>
-      </c>
-      <c r="H25" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>0</v>
+      </c>
+      <c r="I25" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>46</v>
       </c>
       <c r="B26" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C26" t="s">
         <v>169</v>
@@ -1745,24 +1833,27 @@
         <v>47</v>
       </c>
       <c r="E26" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F26" t="s">
         <v>175</v>
       </c>
       <c r="G26">
-        <v>1</v>
-      </c>
-      <c r="H26" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>48</v>
       </c>
       <c r="B27" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C27" t="s">
         <v>169</v>
@@ -1771,7 +1862,7 @@
         <v>49</v>
       </c>
       <c r="E27" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F27" t="s">
         <v>175</v>
@@ -1779,16 +1870,19 @@
       <c r="G27">
         <v>1</v>
       </c>
-      <c r="H27" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>50</v>
       </c>
       <c r="B28" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C28" t="s">
         <v>169</v>
@@ -1805,16 +1899,19 @@
       <c r="G28">
         <v>1</v>
       </c>
-      <c r="H28" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H28">
+        <v>0</v>
+      </c>
+      <c r="I28" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>52</v>
       </c>
       <c r="B29" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C29" t="s">
         <v>169</v>
@@ -1826,21 +1923,24 @@
         <v>163</v>
       </c>
       <c r="F29" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G29">
         <v>1</v>
       </c>
-      <c r="H29" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H29">
+        <v>0</v>
+      </c>
+      <c r="I29" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>54</v>
       </c>
       <c r="B30" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C30" t="s">
         <v>169</v>
@@ -1849,7 +1949,7 @@
         <v>55</v>
       </c>
       <c r="E30" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F30" t="s">
         <v>175</v>
@@ -1857,16 +1957,19 @@
       <c r="G30">
         <v>1</v>
       </c>
-      <c r="H30" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H30">
+        <v>1</v>
+      </c>
+      <c r="I30" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>56</v>
       </c>
       <c r="B31" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C31" t="s">
         <v>169</v>
@@ -1878,21 +1981,24 @@
         <v>163</v>
       </c>
       <c r="F31" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G31">
         <v>1</v>
       </c>
-      <c r="H31" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H31">
+        <v>0</v>
+      </c>
+      <c r="I31" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>58</v>
       </c>
       <c r="B32" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C32" t="s">
         <v>169</v>
@@ -1904,21 +2010,24 @@
         <v>163</v>
       </c>
       <c r="F32" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G32">
         <v>1</v>
       </c>
-      <c r="H32" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H32">
+        <v>0</v>
+      </c>
+      <c r="I32" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>60</v>
       </c>
       <c r="B33" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C33" t="s">
         <v>170</v>
@@ -1930,21 +2039,24 @@
         <v>163</v>
       </c>
       <c r="F33" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="G33">
         <v>1</v>
       </c>
-      <c r="H33" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H33">
+        <v>0</v>
+      </c>
+      <c r="I33" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>62</v>
       </c>
       <c r="B34" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C34" t="s">
         <v>170</v>
@@ -1958,16 +2070,19 @@
       <c r="G34">
         <v>0</v>
       </c>
-      <c r="H34" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H34">
+        <v>0</v>
+      </c>
+      <c r="I34" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>64</v>
       </c>
       <c r="B35" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C35" t="s">
         <v>170</v>
@@ -1976,7 +2091,7 @@
         <v>65</v>
       </c>
       <c r="E35" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F35" t="s">
         <v>176</v>
@@ -1984,16 +2099,19 @@
       <c r="G35">
         <v>1</v>
       </c>
-      <c r="H35" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H35">
+        <v>1</v>
+      </c>
+      <c r="I35" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>66</v>
       </c>
       <c r="B36" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C36" t="s">
         <v>170</v>
@@ -2002,7 +2120,7 @@
         <v>67</v>
       </c>
       <c r="E36" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F36" t="s">
         <v>176</v>
@@ -2010,16 +2128,19 @@
       <c r="G36">
         <v>1</v>
       </c>
-      <c r="H36" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H36">
+        <v>1</v>
+      </c>
+      <c r="I36" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>68</v>
       </c>
       <c r="B37" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C37" t="s">
         <v>170</v>
@@ -2028,7 +2149,7 @@
         <v>69</v>
       </c>
       <c r="E37" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F37" t="s">
         <v>179</v>
@@ -2036,16 +2157,19 @@
       <c r="G37">
         <v>1</v>
       </c>
-      <c r="H37" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H37">
+        <v>1</v>
+      </c>
+      <c r="I37" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>70</v>
       </c>
       <c r="B38" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C38" t="s">
         <v>170</v>
@@ -2054,7 +2178,7 @@
         <v>71</v>
       </c>
       <c r="E38" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F38" t="s">
         <v>176</v>
@@ -2062,16 +2186,19 @@
       <c r="G38">
         <v>1</v>
       </c>
-      <c r="H38" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H38">
+        <v>1</v>
+      </c>
+      <c r="I38" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>72</v>
       </c>
       <c r="B39" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C39" t="s">
         <v>170</v>
@@ -2080,7 +2207,7 @@
         <v>73</v>
       </c>
       <c r="E39" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F39" t="s">
         <v>179</v>
@@ -2088,16 +2215,19 @@
       <c r="G39">
         <v>1</v>
       </c>
-      <c r="H39" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H39">
+        <v>1</v>
+      </c>
+      <c r="I39" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>74</v>
       </c>
       <c r="B40" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C40" t="s">
         <v>170</v>
@@ -2106,7 +2236,7 @@
         <v>75</v>
       </c>
       <c r="E40" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F40" t="s">
         <v>176</v>
@@ -2114,16 +2244,19 @@
       <c r="G40">
         <v>1</v>
       </c>
-      <c r="H40" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H40">
+        <v>1</v>
+      </c>
+      <c r="I40" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>76</v>
       </c>
       <c r="B41" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C41" t="s">
         <v>170</v>
@@ -2132,7 +2265,7 @@
         <v>77</v>
       </c>
       <c r="E41" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F41" t="s">
         <v>179</v>
@@ -2140,16 +2273,19 @@
       <c r="G41">
         <v>1</v>
       </c>
-      <c r="H41" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H41">
+        <v>1</v>
+      </c>
+      <c r="I41" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>78</v>
       </c>
       <c r="B42" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C42" t="s">
         <v>170</v>
@@ -2158,7 +2294,7 @@
         <v>79</v>
       </c>
       <c r="E42" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F42" t="s">
         <v>176</v>
@@ -2166,16 +2302,19 @@
       <c r="G42">
         <v>1</v>
       </c>
-      <c r="H42" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H42">
+        <v>1</v>
+      </c>
+      <c r="I42" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>80</v>
       </c>
       <c r="B43" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C43" t="s">
         <v>170</v>
@@ -2184,7 +2323,7 @@
         <v>81</v>
       </c>
       <c r="E43" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F43" t="s">
         <v>179</v>
@@ -2192,16 +2331,19 @@
       <c r="G43">
         <v>1</v>
       </c>
-      <c r="H43" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H43">
+        <v>1</v>
+      </c>
+      <c r="I43" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>82</v>
       </c>
       <c r="B44" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C44" t="s">
         <v>170</v>
@@ -2210,7 +2352,7 @@
         <v>83</v>
       </c>
       <c r="E44" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F44" t="s">
         <v>176</v>
@@ -2218,16 +2360,19 @@
       <c r="G44">
         <v>1</v>
       </c>
-      <c r="H44" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H44">
+        <v>1</v>
+      </c>
+      <c r="I44" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>84</v>
       </c>
       <c r="B45" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C45" t="s">
         <v>170</v>
@@ -2236,7 +2381,7 @@
         <v>85</v>
       </c>
       <c r="E45" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F45" t="s">
         <v>179</v>
@@ -2244,16 +2389,19 @@
       <c r="G45">
         <v>1</v>
       </c>
-      <c r="H45" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H45">
+        <v>1</v>
+      </c>
+      <c r="I45" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>86</v>
       </c>
       <c r="B46" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C46" t="s">
         <v>170</v>
@@ -2262,7 +2410,7 @@
         <v>87</v>
       </c>
       <c r="E46" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F46" t="s">
         <v>176</v>
@@ -2270,16 +2418,19 @@
       <c r="G46">
         <v>1</v>
       </c>
-      <c r="H46" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H46">
+        <v>1</v>
+      </c>
+      <c r="I46" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>88</v>
       </c>
       <c r="B47" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C47" t="s">
         <v>170</v>
@@ -2288,7 +2439,7 @@
         <v>89</v>
       </c>
       <c r="E47" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F47" t="s">
         <v>179</v>
@@ -2296,16 +2447,19 @@
       <c r="G47">
         <v>1</v>
       </c>
-      <c r="H47" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H47">
+        <v>1</v>
+      </c>
+      <c r="I47" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>90</v>
       </c>
       <c r="B48" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C48" t="s">
         <v>170</v>
@@ -2314,7 +2468,7 @@
         <v>91</v>
       </c>
       <c r="E48" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="F48" t="s">
         <v>176</v>
@@ -2322,16 +2476,19 @@
       <c r="G48">
         <v>1</v>
       </c>
-      <c r="H48" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H48">
+        <v>1</v>
+      </c>
+      <c r="I48" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>92</v>
       </c>
       <c r="B49" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C49" t="s">
         <v>170</v>
@@ -2340,7 +2497,7 @@
         <v>93</v>
       </c>
       <c r="E49" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F49" t="s">
         <v>176</v>
@@ -2348,16 +2505,19 @@
       <c r="G49">
         <v>1</v>
       </c>
-      <c r="H49" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H49">
+        <v>1</v>
+      </c>
+      <c r="I49" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>94</v>
       </c>
       <c r="B50" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C50" t="s">
         <v>170</v>
@@ -2366,7 +2526,7 @@
         <v>95</v>
       </c>
       <c r="E50" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F50" t="s">
         <v>176</v>
@@ -2374,11 +2534,14 @@
       <c r="G50">
         <v>1</v>
       </c>
-      <c r="H50" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H50">
+        <v>1</v>
+      </c>
+      <c r="I50" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>96</v>
       </c>
@@ -2394,11 +2557,14 @@
       <c r="G51">
         <v>0</v>
       </c>
-      <c r="H51" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H51">
+        <v>0</v>
+      </c>
+      <c r="I51" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>98</v>
       </c>
@@ -2411,11 +2577,14 @@
       <c r="G52">
         <v>0</v>
       </c>
-      <c r="H52" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H52">
+        <v>0</v>
+      </c>
+      <c r="I52" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>100</v>
       </c>
@@ -2428,11 +2597,14 @@
       <c r="G53">
         <v>0</v>
       </c>
-      <c r="H53" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H53">
+        <v>0</v>
+      </c>
+      <c r="I53" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>102</v>
       </c>
@@ -2445,11 +2617,14 @@
       <c r="G54">
         <v>0</v>
       </c>
-      <c r="H54" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H54">
+        <v>0</v>
+      </c>
+      <c r="I54" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>104</v>
       </c>
@@ -2465,11 +2640,14 @@
       <c r="G55">
         <v>0</v>
       </c>
-      <c r="H55" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H55">
+        <v>0</v>
+      </c>
+      <c r="I55" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>106</v>
       </c>
@@ -2482,11 +2660,14 @@
       <c r="G56">
         <v>0</v>
       </c>
-      <c r="H56" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>108</v>
       </c>
@@ -2502,11 +2683,14 @@
       <c r="G57">
         <v>0</v>
       </c>
-      <c r="H57" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H57">
+        <v>0</v>
+      </c>
+      <c r="I57" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>110</v>
       </c>
@@ -2519,11 +2703,14 @@
       <c r="G58">
         <v>0</v>
       </c>
-      <c r="H58" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H58">
+        <v>0</v>
+      </c>
+      <c r="I58" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>112</v>
       </c>
@@ -2539,11 +2726,14 @@
       <c r="G59">
         <v>0</v>
       </c>
-      <c r="H59" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H59">
+        <v>0</v>
+      </c>
+      <c r="I59" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>114</v>
       </c>
@@ -2556,11 +2746,14 @@
       <c r="G60">
         <v>0</v>
       </c>
-      <c r="H60" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H60">
+        <v>0</v>
+      </c>
+      <c r="I60" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>116</v>
       </c>
@@ -2576,11 +2769,14 @@
       <c r="G61">
         <v>0</v>
       </c>
-      <c r="H61" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H61">
+        <v>0</v>
+      </c>
+      <c r="I61" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>118</v>
       </c>
@@ -2593,11 +2789,14 @@
       <c r="G62">
         <v>0</v>
       </c>
-      <c r="H62" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H62">
+        <v>0</v>
+      </c>
+      <c r="I62" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>120</v>
       </c>
@@ -2613,11 +2812,14 @@
       <c r="G63">
         <v>0</v>
       </c>
-      <c r="H63" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H63">
+        <v>0</v>
+      </c>
+      <c r="I63" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>122</v>
       </c>
@@ -2630,11 +2832,14 @@
       <c r="G64">
         <v>0</v>
       </c>
-      <c r="H64" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H64">
+        <v>0</v>
+      </c>
+      <c r="I64" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>124</v>
       </c>
@@ -2650,11 +2855,14 @@
       <c r="G65">
         <v>0</v>
       </c>
-      <c r="H65" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H65">
+        <v>0</v>
+      </c>
+      <c r="I65" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>126</v>
       </c>
@@ -2667,11 +2875,14 @@
       <c r="G66">
         <v>0</v>
       </c>
-      <c r="H66" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H66">
+        <v>0</v>
+      </c>
+      <c r="I66" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>128</v>
       </c>
@@ -2687,11 +2898,14 @@
       <c r="G67">
         <v>0</v>
       </c>
-      <c r="H67" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H67">
+        <v>0</v>
+      </c>
+      <c r="I67" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>130</v>
       </c>
@@ -2704,11 +2918,14 @@
       <c r="G68">
         <v>0</v>
       </c>
-      <c r="H68" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H68">
+        <v>0</v>
+      </c>
+      <c r="I68" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>132</v>
       </c>
@@ -2724,11 +2941,14 @@
       <c r="G69">
         <v>0</v>
       </c>
-      <c r="H69" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H69">
+        <v>0</v>
+      </c>
+      <c r="I69" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>134</v>
       </c>
@@ -2741,11 +2961,14 @@
       <c r="G70">
         <v>0</v>
       </c>
-      <c r="H70" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H70">
+        <v>0</v>
+      </c>
+      <c r="I70" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>136</v>
       </c>
@@ -2758,11 +2981,14 @@
       <c r="G71">
         <v>0</v>
       </c>
-      <c r="H71" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H71">
+        <v>0</v>
+      </c>
+      <c r="I71" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>138</v>
       </c>
@@ -2775,11 +3001,14 @@
       <c r="G72">
         <v>0</v>
       </c>
-      <c r="H72" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H72">
+        <v>0</v>
+      </c>
+      <c r="I72" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>140</v>
       </c>
@@ -2795,11 +3024,14 @@
       <c r="G73">
         <v>0</v>
       </c>
-      <c r="H73" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H73">
+        <v>0</v>
+      </c>
+      <c r="I73" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>142</v>
       </c>
@@ -2812,11 +3044,14 @@
       <c r="G74">
         <v>0</v>
       </c>
-      <c r="H74" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H74">
+        <v>0</v>
+      </c>
+      <c r="I74" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>144</v>
       </c>
@@ -2832,11 +3067,14 @@
       <c r="G75">
         <v>0</v>
       </c>
-      <c r="H75" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H75">
+        <v>0</v>
+      </c>
+      <c r="I75" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>146</v>
       </c>
@@ -2849,11 +3087,14 @@
       <c r="G76">
         <v>0</v>
       </c>
-      <c r="H76" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H76">
+        <v>0</v>
+      </c>
+      <c r="I76" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>148</v>
       </c>
@@ -2866,11 +3107,14 @@
       <c r="G77">
         <v>0</v>
       </c>
-      <c r="H77" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H77">
+        <v>0</v>
+      </c>
+      <c r="I77" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>150</v>
       </c>
@@ -2883,11 +3127,14 @@
       <c r="G78">
         <v>0</v>
       </c>
-      <c r="H78" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H78">
+        <v>0</v>
+      </c>
+      <c r="I78" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>152</v>
       </c>
@@ -2900,11 +3147,14 @@
       <c r="G79">
         <v>0</v>
       </c>
-      <c r="H79" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H79">
+        <v>0</v>
+      </c>
+      <c r="I79" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>154</v>
       </c>
@@ -2917,11 +3167,14 @@
       <c r="G80">
         <v>0</v>
       </c>
-      <c r="H80" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.3">
+      <c r="H80">
+        <v>0</v>
+      </c>
+      <c r="I80" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>156</v>
       </c>
@@ -2934,18 +3187,15 @@
       <c r="G81">
         <v>0</v>
       </c>
-      <c r="H81" t="s">
-        <v>184</v>
+      <c r="H81">
+        <v>0</v>
+      </c>
+      <c r="I81" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H81" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters>
-        <filter val="categorical"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:I81" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>